<commit_message>
adding lab 1 changes and rubric
</commit_message>
<xml_diff>
--- a/docs/project/Lab_01_rubric.xlsx
+++ b/docs/project/Lab_01_rubric.xlsx
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -703,7 +703,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8604CA67-57A5-BA4E-8D98-9A6B26E901C2}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.83203125" style="11" customWidth="1"/>
@@ -716,259 +716,331 @@
     <col min="8" max="16384" width="10.83203125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Section</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Item</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Points</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Satisfactory</t>
+        </is>
+      </c>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.1 WBNS Background</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What is the motivation for this study? Answered using information from the WBNS sources</t>
+        </is>
+      </c>
+      <c r="C2" s="4">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sections</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grade</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Possible</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="51" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.1 WBNS Background</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How could an information sheet on WBNS components help change policy? Answered using information from the WBNS sources</t>
+        </is>
+      </c>
+      <c r="C3" s="4">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.1 WBNS Background</t>
+        </is>
+      </c>
+      <c r="G3" s="3">
+        <f>SUMIF($D$2:$D$4,TRUE,$C$2:$C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="10">
+        <f>SUM($C$2:$C$4)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.1 WBNS Background</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why is it important to study basic needs? Answered using information from the WBNS sources</t>
+        </is>
+      </c>
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.2 File Organization</t>
+        </is>
+      </c>
+      <c r="G4" s="3">
+        <f>SUMIF($D$5:$D$6,TRUE,$C$5:$C$6)</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="10">
+        <f>SUM($C$5:$C$6)</f>
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.2 File Organization</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Working directory displayed using here(), with the output visible in the .html</t>
+        </is>
+      </c>
+      <c r="C5" s="11">
+        <v>1</v>
+      </c>
+      <c r="D5" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.3 Data Access</t>
+        </is>
+      </c>
+      <c r="G5" s="3">
+        <f>SUMIF($D$7:$D$7,TRUE,$C$7:$C$7)</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="10">
+        <f>SUM($C$7:$C$7)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" ht="51" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.2 File Organization</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Screenshot of the course folder showing the .Rproj file in the top level of the course folder, not inside a subfolder</t>
+        </is>
+      </c>
+      <c r="C6" s="11">
+        <v>1</v>
+      </c>
+      <c r="D6" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.4 Load &amp; Rename Data</t>
+        </is>
+      </c>
+      <c r="G6" s="3">
+        <f>SUMIF($D$8:$D$11,TRUE,$C$8:$C$11)</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="10">
+        <f>SUM($C$8:$C$11)</f>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="7" ht="51" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.3 Data Access</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Downloaded data saved inside data_project (data_raw recommended), shown by the folder screenshot or the file path in the loading code</t>
+        </is>
+      </c>
+      <c r="C7" s="4">
+        <v>1</v>
+      </c>
+      <c r="D7" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.5 Project Question</t>
+        </is>
+      </c>
+      <c r="G7" s="3">
+        <f>SUMIF($D$12:$D$13,TRUE,$C$12:$C$13)</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="10">
+        <f>SUM($C$12:$C$13)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.4 Load &amp; Rename Data</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Uses a correct function for .rda files (e.g., load())</t>
+        </is>
+      </c>
+      <c r="C8" s="11">
+        <v>1</v>
+      </c>
+      <c r="D8" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.6 Data Formatting</t>
+        </is>
+      </c>
+      <c r="G8" s="3">
+        <f>SUMIF($D$14:$D$16,TRUE,$C$14:$C$16)</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="10">
+        <f>SUM($C$14:$C$16)</f>
         <v>3</v>
       </c>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="4">
-        <v>1</v>
-      </c>
-      <c r="D2" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="4">
-        <v>1</v>
-      </c>
-      <c r="D3" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" s="3">
-        <f>SUM(IF($D$2=FALSE,0,1)*$C$2,IF($D$3=FALSE,0,1)*$C$3,IF($D$4=FALSE,0,1)*$C$4,IF($D$5=FALSE,0,1)*$C$5)</f>
-        <v>0</v>
-      </c>
-      <c r="H3" s="10">
-        <f>SUM($C$2:$C$5)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="4">
-        <v>1</v>
-      </c>
-      <c r="D4" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="3">
-        <f>SUM(IF($D$6=FALSE,0,1)*$C$6,IF($D$7=FALSE,0,1)*$C$7)</f>
-        <v>0</v>
-      </c>
-      <c r="H4" s="10">
-        <f>SUM($C$6:$C$7)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="4">
-        <v>1</v>
-      </c>
-      <c r="D5" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="3">
-        <f>SUM(IF($D$8=FALSE,0,1)*$C$8,IF($D$9=FALSE,0,1)*$C$9)</f>
-        <v>0</v>
-      </c>
-      <c r="H5" s="10">
-        <f>SUM($C$8:$C$9)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="11">
-        <v>1</v>
-      </c>
-      <c r="D6" s="12" t="b">
-        <v>0</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="3">
-        <f>SUM(IF($D$10=FALSE,0,1)*$C$10,IF($D$11=FALSE,0,1)*$C$11,IF($D$12=FALSE,0,1)*$C$12)</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="10">
-        <f>SUM($C$10:$C$12)</f>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.4 Load &amp; Rename Data</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">File path built with here() and points to the .rda file inside the project's data folder</t>
+        </is>
+      </c>
+      <c r="C9" s="11">
+        <v>1</v>
+      </c>
+      <c r="D9" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.7 Save Processed Data</t>
+        </is>
+      </c>
+      <c r="G9" s="3">
+        <f>SUMIF($D$17:$D$19,TRUE,$C$17:$C$19)</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="10">
+        <f>SUM($C$17:$C$19)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="11">
-        <v>1</v>
-      </c>
-      <c r="D7" s="12" t="b">
-        <v>0</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="G7" s="3">
-        <f>SUM(IF($D$13=FALSE,0,1)*$C$13,IF($D$14=FALSE,0,1)*$C$14)</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="10">
-        <f>SUM($C$13:$C$14)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="4">
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.4 Load &amp; Rename Data</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loaded object saved under a clean, intuitive dataset name (e.g., wbns_data)</t>
+        </is>
+      </c>
+      <c r="C10" s="11">
+        <v>1</v>
+      </c>
+      <c r="D10" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">General / Document Quality</t>
+        </is>
+      </c>
+      <c r="G10" s="3">
+        <f>SUMIF($D$20:$D$23,TRUE,$C$20:$C$23)</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="10">
+        <f>SUM($C$20:$C$23)</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.4 Load &amp; Rename Data</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code is visible in the .html (not just output)</t>
+        </is>
+      </c>
+      <c r="C11" s="11">
         <v>0.5</v>
       </c>
-      <c r="D8" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="G8" s="3">
-        <f>SUM(IF($D$15=FALSE,0,1)*$C$15,IF($D$16=FALSE,0,1)*$C$16,IF($D$17=FALSE,0,1)*$C$17)</f>
-        <v>0</v>
-      </c>
-      <c r="H8" s="10">
-        <f>SUM($C$15:$C$17)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="D9" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="G9" s="3">
-        <f>SUM(IF($D$18=FALSE,0,1)*$C$18,IF($D$19=FALSE,0,1)*$C$19,IF($D$20=FALSE,0,1)*$C$20)</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="10">
-        <f>SUM($C$18:$C$20)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D10" s="12" t="b">
-        <v>0</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="G10" s="3">
-        <f>SUM(IF($D$21=FALSE,0,1)*$C$21,IF($D$22=FALSE,0,1)*$C$22,IF($D$23=FALSE,0,1)*$C$23,IF($D$24=FALSE,0,1)*$C$24)</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="10">
-        <f>SUM($C$21:$C$24)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="11">
-        <v>1</v>
-      </c>
       <c r="D11" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="F11" s="13" t="s">
-        <v>7</v>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total</t>
+        </is>
       </c>
       <c r="G11" s="14">
         <f>SUM(G3:G10)</f>
@@ -976,155 +1048,199 @@
       </c>
       <c r="H11" s="15">
         <f>SUM(H3:H10)</f>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="11">
+        <v>20.0</v>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.5 Project Question</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Project option number (1, 2, or 3) stated</t>
+        </is>
+      </c>
+      <c r="C12" s="4">
+        <v>1</v>
+      </c>
+      <c r="D12" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.5 Project Question</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Project question written out (if custom, note that it was approved by Nicky)</t>
+        </is>
+      </c>
+      <c r="C13" s="4">
+        <v>1</v>
+      </c>
+      <c r="D13" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.6 Data Formatting</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Provided code uses your own dataset names (not old_df/new_df)</t>
+        </is>
+      </c>
+      <c r="C14" s="11">
+        <v>1</v>
+      </c>
+      <c r="D14" s="12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.6 Data Formatting</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code runs without error</t>
+        </is>
+      </c>
+      <c r="C15" s="11">
+        <v>1</v>
+      </c>
+      <c r="D15" s="12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.6 Data Formatting</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">glimpse() output is visible and shows category labels with no (1)-style prefixes</t>
+        </is>
+      </c>
+      <c r="C16" s="11">
+        <v>1</v>
+      </c>
+      <c r="D16" s="12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.7 Save Processed Data</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R code saves the cleaned dataset as a new .rds file (raw data left untouched)</t>
+        </is>
+      </c>
+      <c r="C17" s="4">
+        <v>1</v>
+      </c>
+      <c r="D17" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.7 Save Processed Data</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">File saved into data_project/data_processed</t>
+        </is>
+      </c>
+      <c r="C18" s="4">
+        <v>1</v>
+      </c>
+      <c r="D18" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.7 Save Processed Data</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Screenshot showing the new .rds file inside data_project/data_processed</t>
+        </is>
+      </c>
+      <c r="C19" s="4">
+        <v>1</v>
+      </c>
+      <c r="D19" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">General / Document Quality</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Started from the provided editing file; no headings, tasks, or directions deleted</t>
+        </is>
+      </c>
+      <c r="C20" s="11">
         <v>0.5</v>
       </c>
-      <c r="D12" s="12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" s="4">
-        <v>1</v>
-      </c>
-      <c r="D13" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="4">
-        <v>1</v>
-      </c>
-      <c r="D14" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D15" s="12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="D16" s="12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A17" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" s="11">
-        <v>1</v>
-      </c>
-      <c r="D17" s="12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="4">
-        <v>1</v>
-      </c>
-      <c r="D18" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C19" s="4">
-        <v>1</v>
-      </c>
-      <c r="D19" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C20" s="4">
-        <v>1</v>
-      </c>
-      <c r="D20" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A21" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>34</v>
+      <c r="D20" s="12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">General / Document Quality</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">File renders without errors</t>
+        </is>
       </c>
       <c r="C21" s="11">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D21" s="12" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>35</v>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">General / Document Quality</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Both files follow the naming convention: lastname_firstinit_lab_01.qmd and lastname_firstinit_lab_01.html</t>
+        </is>
       </c>
       <c r="C22" s="11">
         <v>0.5</v>
@@ -1133,31 +1249,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A23" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>36</v>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">General / Document Quality</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code is readable and organized (no leftover scratch code)</t>
+        </is>
       </c>
       <c r="C23" s="11">
         <v>0.5</v>
       </c>
       <c r="D23" s="12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C24" s="11">
-        <v>0.5</v>
-      </c>
-      <c r="D24" s="12" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
adding lab 2 due date
</commit_message>
<xml_diff>
--- a/docs/project/Lab_01_rubric.xlsx
+++ b/docs/project/Lab_01_rubric.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ohsuitg-my.sharepoint.com/personal/wakim_ohsu_edu/Documents/Teaching/Classes/PUBH_523_26Su/PUBH_523_26Su_site/project/"/>
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4" fullCalcOnLoad="1"/>
+  <calcPr calcId="191028" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="38">
   <si>
     <t>Section</t>
   </si>
@@ -50,6 +50,12 @@
     <t>Satisfactory</t>
   </si>
   <si>
+    <t>1.1 WBNS Background</t>
+  </si>
+  <si>
+    <t>What is the motivation for this study? Answered using information from the WBNS sources</t>
+  </si>
+  <si>
     <t>Sections</t>
   </si>
   <si>
@@ -59,107 +65,98 @@
     <t>Possible</t>
   </si>
   <si>
+    <t>How could an information sheet on WBNS components help change policy? Answered using information from the WBNS sources</t>
+  </si>
+  <si>
+    <t>Why is it important to study basic needs? Answered using information from the WBNS sources</t>
+  </si>
+  <si>
+    <t>1.2 File Organization</t>
+  </si>
+  <si>
+    <t>Working directory displayed using here(), with the output visible in the .html</t>
+  </si>
+  <si>
+    <t>1.3 Data Access</t>
+  </si>
+  <si>
+    <t>Screenshot of the course folder showing the .Rproj file in the top level of the course folder, not inside a subfolder</t>
+  </si>
+  <si>
+    <t>1.4 Load &amp; Rename Data</t>
+  </si>
+  <si>
+    <t>Downloaded data saved inside data_project (data_raw recommended), shown by the folder screenshot or the file path in the loading code</t>
+  </si>
+  <si>
+    <t>1.5 Project Question</t>
+  </si>
+  <si>
+    <t>Uses a correct function for .rda files (e.g., load())</t>
+  </si>
+  <si>
+    <t>1.6 Data Formatting</t>
+  </si>
+  <si>
+    <t>File path built with here() and points to the .rda file inside the project's data folder</t>
+  </si>
+  <si>
+    <t>1.7 Save Processed Data</t>
+  </si>
+  <si>
+    <t>Loaded object saved under a clean, intuitive dataset name (e.g., wbns_data)</t>
+  </si>
+  <si>
+    <t>General / Document Quality</t>
+  </si>
+  <si>
+    <t>Code is visible in the .html (not just output)</t>
+  </si>
+  <si>
     <t>Total</t>
   </si>
   <si>
-    <t>1.1 WBNS Background</t>
-  </si>
-  <si>
-    <t>Read the Urban Institute's WBNS page and at least 4 pages of related published material (including the 'From Safety Net to Solid Ground' initiative)</t>
-  </si>
-  <si>
-    <t>Answered: What is the motivation for this study?</t>
-  </si>
-  <si>
-    <t>Answered: How could an information sheet on WBNS components help change policy?</t>
-  </si>
-  <si>
-    <t>Answered: Why is it important to study basic needs?</t>
-  </si>
-  <si>
-    <t>1.2 File Organization</t>
-  </si>
-  <si>
-    <t>Working directory displayed in the .qmd using the here package / here() function, with output visible</t>
-  </si>
-  <si>
-    <t>Screenshot included showing folder organization with the .Rproj file in the correct (top-level project) location</t>
-  </si>
-  <si>
-    <t>1.3 Data Access</t>
-  </si>
-  <si>
-    <t>Data downloaded from ICPSR and placed inside a data folder within the project directory</t>
-  </si>
-  <si>
-    <t>Evidence the User Guide was reviewed (e.g., correct variable names/usage downstream)</t>
-  </si>
-  <si>
-    <t>1.4 Load &amp; Rename Data</t>
-  </si>
-  <si>
-    <t>Data loaded into R using a correct method for .rda files and a correct file path built with here()</t>
-  </si>
-  <si>
-    <t>Loaded object renamed to a clean, intuitive dataset name</t>
-  </si>
-  <si>
-    <t>Code shown/visible in the .qmd (not just output)</t>
-  </si>
-  <si>
-    <t>1.5 Project Question</t>
-  </si>
-  <si>
-    <t>One of the 3 project options selected, with the option number stated explicitly</t>
-  </si>
-  <si>
-    <t>1.6 Data Formatting</t>
-  </si>
-  <si>
-    <t>Provided mutate()/across() code adapted correctly with student's actual old_df/new_df names</t>
-  </si>
-  <si>
-    <t>Code runs without error and parentheses/leading numeric codes are removed from factor level labels</t>
-  </si>
-  <si>
-    <t>glimpse() used afterward to verify the parentheses are gone, with output visible</t>
-  </si>
-  <si>
-    <t>1.7 Save Processed Data</t>
-  </si>
-  <si>
-    <t>R code used to save the cleaned dataset as a new .Rda file (separate from raw data)</t>
-  </si>
-  <si>
-    <t>File saved into the correct data subfolder per the project's file structure</t>
-  </si>
-  <si>
-    <t>Screenshot included showing the new .Rda file inside the data folder</t>
-  </si>
-  <si>
-    <t>General / Document Quality</t>
-  </si>
-  <si>
-    <t>Editing file is the correct, unmodified .qmd template -- no instructional text/sections deleted</t>
-  </si>
-  <si>
-    <t>File renders (knits) without errors</t>
-  </si>
-  <si>
-    <t>File follows naming convention: lastname_firstinit_lab_01.qmd</t>
-  </si>
-  <si>
-    <t>Code is reasonably readable/organized (chunks labeled, no leftover scratch code)</t>
-  </si>
-  <si>
-    <t>Question written out clearly (or, if custom, evidence it was pre-approved)</t>
+    <t>Project option number (1, 2, or 3) stated</t>
+  </si>
+  <si>
+    <t>Project question written out (if custom, note that it was approved by Nicky)</t>
+  </si>
+  <si>
+    <t>Provided code uses your own dataset names (not old_df/new_df)</t>
+  </si>
+  <si>
+    <t>Code runs without error</t>
+  </si>
+  <si>
+    <t>glimpse() output is visible and shows category labels with no (1)-style prefixes</t>
+  </si>
+  <si>
+    <t>R code saves the cleaned dataset as a new .rds file (raw data left untouched)</t>
+  </si>
+  <si>
+    <t>File saved into data_project/data_processed</t>
+  </si>
+  <si>
+    <t>Screenshot showing the new .rds file inside data_project/data_processed</t>
+  </si>
+  <si>
+    <t>Started from the provided editing file; no headings, tasks, or directions deleted</t>
+  </si>
+  <si>
+    <t>File renders without errors</t>
+  </si>
+  <si>
+    <t>Both files follow the naming convention: lastname_firstinit_lab_01.qmd and lastname_firstinit_lab_01.html</t>
+  </si>
+  <si>
+    <t>Code is readable and organized (no leftover scratch code)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -704,51 +701,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8604CA67-57A5-BA4E-8D98-9A6B26E901C2}">
   <dimension ref="A1:H23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" style="11" customWidth="1"/>
+    <col min="1" max="1" width="25.875" style="11" customWidth="1"/>
     <col min="2" max="2" width="57" style="11" customWidth="1"/>
     <col min="3" max="3" width="8" style="11" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" style="11" customWidth="1"/>
-    <col min="5" max="5" width="8.33203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.625" style="11" customWidth="1"/>
+    <col min="5" max="5" width="8.375" style="3" customWidth="1"/>
     <col min="6" max="6" width="26.5" style="3" customWidth="1"/>
-    <col min="7" max="7" width="11.1640625" style="3" customWidth="1"/>
-    <col min="8" max="16384" width="10.83203125" style="3"/>
+    <col min="7" max="7" width="11.125" style="3" customWidth="1"/>
+    <col min="8" max="16384" width="10.875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Section</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Item</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Points</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Satisfactory</t>
-        </is>
+    <row r="1" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="E1" s="2"/>
     </row>
-    <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.1 WBNS Background</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">What is the motivation for this study? Answered using information from the WBNS sources</t>
-        </is>
+    <row r="2" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>5</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
@@ -756,32 +741,22 @@
       <c r="D2" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sections</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Grade</t>
-        </is>
-      </c>
-      <c r="H2" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Possible</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="51" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.1 WBNS Background</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How could an information sheet on WBNS components help change policy? Answered using information from the WBNS sources</t>
-        </is>
+      <c r="F2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="51" customHeight="1">
+      <c r="A3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="C3" s="4">
         <v>1</v>
@@ -789,10 +764,8 @@
       <c r="D3" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.1 WBNS Background</t>
-        </is>
+      <c r="F3" s="9" t="s">
+        <v>4</v>
       </c>
       <c r="G3" s="3">
         <f>SUMIF($D$2:$D$4,TRUE,$C$2:$C$4)</f>
@@ -803,16 +776,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.1 WBNS Background</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Why is it important to study basic needs? Answered using information from the WBNS sources</t>
-        </is>
+    <row r="4" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="C4" s="4">
         <v>1</v>
@@ -820,10 +789,8 @@
       <c r="D4" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.2 File Organization</t>
-        </is>
+      <c r="F4" s="9" t="s">
+        <v>11</v>
       </c>
       <c r="G4" s="3">
         <f>SUMIF($D$5:$D$6,TRUE,$C$5:$C$6)</f>
@@ -834,16 +801,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.2 File Organization</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Working directory displayed using here(), with the output visible in the .html</t>
-        </is>
+    <row r="5" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A5" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>12</v>
       </c>
       <c r="C5" s="11">
         <v>1</v>
@@ -851,10 +814,8 @@
       <c r="D5" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.3 Data Access</t>
-        </is>
+      <c r="F5" s="9" t="s">
+        <v>13</v>
       </c>
       <c r="G5" s="3">
         <f>SUMIF($D$7:$D$7,TRUE,$C$7:$C$7)</f>
@@ -865,16 +826,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" ht="51" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.2 File Organization</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Screenshot of the course folder showing the .Rproj file in the top level of the course folder, not inside a subfolder</t>
-        </is>
+    <row r="6" spans="1:8" ht="51" customHeight="1">
+      <c r="A6" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>14</v>
       </c>
       <c r="C6" s="11">
         <v>1</v>
@@ -882,10 +839,8 @@
       <c r="D6" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.4 Load &amp; Rename Data</t>
-        </is>
+      <c r="F6" s="9" t="s">
+        <v>15</v>
       </c>
       <c r="G6" s="3">
         <f>SUMIF($D$8:$D$11,TRUE,$C$8:$C$11)</f>
@@ -896,16 +851,12 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="7" ht="51" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.3 Data Access</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Downloaded data saved inside data_project (data_raw recommended), shown by the folder screenshot or the file path in the loading code</t>
-        </is>
+    <row r="7" spans="1:8" ht="51" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="C7" s="4">
         <v>1</v>
@@ -913,10 +864,8 @@
       <c r="D7" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.5 Project Question</t>
-        </is>
+      <c r="F7" s="9" t="s">
+        <v>17</v>
       </c>
       <c r="G7" s="3">
         <f>SUMIF($D$12:$D$13,TRUE,$C$12:$C$13)</f>
@@ -927,16 +876,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.4 Load &amp; Rename Data</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Uses a correct function for .rda files (e.g., load())</t>
-        </is>
+    <row r="8" spans="1:8" ht="17.100000000000001" customHeight="1">
+      <c r="A8" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>18</v>
       </c>
       <c r="C8" s="11">
         <v>1</v>
@@ -944,10 +889,8 @@
       <c r="D8" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.6 Data Formatting</t>
-        </is>
+      <c r="F8" s="9" t="s">
+        <v>19</v>
       </c>
       <c r="G8" s="3">
         <f>SUMIF($D$14:$D$16,TRUE,$C$14:$C$16)</f>
@@ -958,16 +901,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.4 Load &amp; Rename Data</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">File path built with here() and points to the .rda file inside the project's data folder</t>
-        </is>
+    <row r="9" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A9" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>20</v>
       </c>
       <c r="C9" s="11">
         <v>1</v>
@@ -975,10 +914,8 @@
       <c r="D9" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.7 Save Processed Data</t>
-        </is>
+      <c r="F9" s="9" t="s">
+        <v>21</v>
       </c>
       <c r="G9" s="3">
         <f>SUMIF($D$17:$D$19,TRUE,$C$17:$C$19)</f>
@@ -989,16 +926,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.4 Load &amp; Rename Data</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Loaded object saved under a clean, intuitive dataset name (e.g., wbns_data)</t>
-        </is>
+    <row r="10" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A10" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>22</v>
       </c>
       <c r="C10" s="11">
         <v>1</v>
@@ -1006,10 +939,8 @@
       <c r="D10" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">General / Document Quality</t>
-        </is>
+      <c r="F10" s="9" t="s">
+        <v>23</v>
       </c>
       <c r="G10" s="3">
         <f>SUMIF($D$20:$D$23,TRUE,$C$20:$C$23)</f>
@@ -1020,16 +951,12 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.4 Load &amp; Rename Data</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Code is visible in the .html (not just output)</t>
-        </is>
+    <row r="11" spans="1:8" ht="17.100000000000001" customHeight="1">
+      <c r="A11" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>24</v>
       </c>
       <c r="C11" s="11">
         <v>0.5</v>
@@ -1037,10 +964,8 @@
       <c r="D11" s="12" t="b">
         <v>0</v>
       </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total</t>
-        </is>
+      <c r="F11" s="13" t="s">
+        <v>25</v>
       </c>
       <c r="G11" s="14">
         <f>SUM(G3:G10)</f>
@@ -1048,19 +973,15 @@
       </c>
       <c r="H11" s="15">
         <f>SUM(H3:H10)</f>
-        <v>20.0</v>
-      </c>
-    </row>
-    <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.5 Project Question</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Project option number (1, 2, or 3) stated</t>
-        </is>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="17.100000000000001" customHeight="1">
+      <c r="A12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="C12" s="4">
         <v>1</v>
@@ -1069,16 +990,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.5 Project Question</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Project question written out (if custom, note that it was approved by Nicky)</t>
-        </is>
+    <row r="13" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="C13" s="4">
         <v>1</v>
@@ -1087,16 +1004,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.6 Data Formatting</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Provided code uses your own dataset names (not old_df/new_df)</t>
-        </is>
+    <row r="14" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A14" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>28</v>
       </c>
       <c r="C14" s="11">
         <v>1</v>
@@ -1105,16 +1018,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.6 Data Formatting</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Code runs without error</t>
-        </is>
+    <row r="15" spans="1:8" ht="17.100000000000001" customHeight="1">
+      <c r="A15" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>29</v>
       </c>
       <c r="C15" s="11">
         <v>1</v>
@@ -1123,16 +1032,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.6 Data Formatting</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">glimpse() output is visible and shows category labels with no (1)-style prefixes</t>
-        </is>
+    <row r="16" spans="1:8" ht="33.950000000000003" customHeight="1">
+      <c r="A16" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>30</v>
       </c>
       <c r="C16" s="11">
         <v>1</v>
@@ -1141,16 +1046,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.7 Save Processed Data</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R code saves the cleaned dataset as a new .rds file (raw data left untouched)</t>
-        </is>
+    <row r="17" spans="1:4" ht="33.950000000000003" customHeight="1">
+      <c r="A17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>31</v>
       </c>
       <c r="C17" s="4">
         <v>1</v>
@@ -1159,16 +1060,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" ht="17" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.7 Save Processed Data</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">File saved into data_project/data_processed</t>
-        </is>
+    <row r="18" spans="1:4" ht="17.100000000000001" customHeight="1">
+      <c r="A18" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>32</v>
       </c>
       <c r="C18" s="4">
         <v>1</v>
@@ -1177,16 +1074,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.7 Save Processed Data</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Screenshot showing the new .rds file inside data_project/data_processed</t>
-        </is>
+    <row r="19" spans="1:4" ht="33.950000000000003" customHeight="1">
+      <c r="A19" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="C19" s="4">
         <v>1</v>
@@ -1195,16 +1088,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">General / Document Quality</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Started from the provided editing file; no headings, tasks, or directions deleted</t>
-        </is>
+    <row r="20" spans="1:4" ht="33.950000000000003" customHeight="1">
+      <c r="A20" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>34</v>
       </c>
       <c r="C20" s="11">
         <v>0.5</v>
@@ -1213,16 +1102,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="17" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">General / Document Quality</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">File renders without errors</t>
-        </is>
+    <row r="21" spans="1:4" ht="17.100000000000001" customHeight="1">
+      <c r="A21" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>35</v>
       </c>
       <c r="C21" s="11">
         <v>1</v>
@@ -1231,16 +1116,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">General / Document Quality</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Both files follow the naming convention: lastname_firstinit_lab_01.qmd and lastname_firstinit_lab_01.html</t>
-        </is>
+    <row r="22" spans="1:4" ht="33.950000000000003" customHeight="1">
+      <c r="A22" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>36</v>
       </c>
       <c r="C22" s="11">
         <v>0.5</v>
@@ -1249,16 +1130,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="17" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">General / Document Quality</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Code is readable and organized (no leftover scratch code)</t>
-        </is>
+    <row r="23" spans="1:4" ht="17.100000000000001" customHeight="1">
+      <c r="A23" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>37</v>
       </c>
       <c r="C23" s="11">
         <v>0.5</v>

</xml_diff>